<commit_message>
event2027: strong reply-all instruction in RFP mail and form
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/public/admin/event2027/files/snu2027_rfp_response_form.xlsx
+++ b/site/public/admin/event2027/files/snu2027_rfp_response_form.xlsx
@@ -622,7 +622,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>작성 방법</t>
@@ -630,7 +630,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>노란 칸만 입력해 주십시오. 파일명을 '회신양식_회사명.xlsx'로 저장해 pm@snubusiness.com 으로 보내 주십시오.</t>
+          <t>노란 칸만 입력해 주십시오. 파일명을 '회신양식_회사명.xlsx'로 저장해, 받으신 메일에 반드시 '전체 회신(Reply All)'으로 보내 주십시오. pm@snubusiness.com 이 빠진 회신은 접수되지 않을 수 있습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
event2027: response form sheet 4 = 8 common checks (hotel setup, show/subcontract, cost split)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/public/admin/event2027/files/snu2027_rfp_response_form.xlsx
+++ b/site/public/admin/event2027/files/snu2027_rfp_response_form.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 참여의사·담당자" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 수행실적" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 투입인력" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 역량·조건" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 공통 확인·조건" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 견적(700명)" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 인원 증감" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 예산 내 차별화" sheetId="8" state="visible" r:id="rId8"/>
@@ -1283,11 +1283,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
@@ -1295,21 +1295,21 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>4. 운영 역량 및 필수 조건</t>
+          <t>4. 공통 확인 8가지 및 필수 조건</t>
         </is>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>서술은 간단히, 상세는 제안서에 기재해 주십시오.</t>
+          <t>모든 업체에 같은 질문을 드립니다. 짧게 답하고, 상세는 제안서 쪽수를 적어 주십시오. 다른 시트에 이미 적은 내용은 '시트 2 참조'처럼 표시해도 됩니다.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>구분</t>
+          <t>공통 확인</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1328,145 +1328,201 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="46" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>프로그램</t>
+          <t>① 참여·일정</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>창립총회 의결·만찬·특별 강연·창립 세리머니·네트워킹을 18:00–21:00 안에 어떻게 배분하는가 (분 단위 개요)</t>
+          <t>2027.4.16(금) 현장 운영 가능 여부와, 11월 제안서(11/6)·PT(11월 둘째 주) 일정 대응 가능 여부</t>
         </is>
       </c>
       <c r="C5" s="8" t="n"/>
       <c r="D5" s="8" t="n"/>
     </row>
-    <row r="6" ht="42" customHeight="1">
+    <row r="6" ht="46" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>프로그램</t>
+          <t>② 실제 실적</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>창립 메시지를 드러내는 오프닝·세리머니 핵심 아이디어 1~2개</t>
+          <t>최근 5년 500~1,000명 규모 갈라·창립기념식·VIP 만찬 중 귀사가 '직접 총괄'한 대표 사례 2~3건 (시트 2에 상세)</t>
         </is>
       </c>
       <c r="C6" s="8" t="n"/>
       <c r="D6" s="8" t="n"/>
     </row>
-    <row r="7" ht="42" customHeight="1">
+    <row r="7" ht="46" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>제작</t>
+          <t>③ 실제 인력</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>무대·AV·영상·디자인 중 사내 제작과 외주 항목 구분 (외주 파트너명)</t>
+          <t>총괄 PM·크리에이티브 디렉터·현장 운영책임자의 이름·직책·대표 실적·투입률 (시트 3에 상세). 제안서 인력과 실제 투입 인력이 같은가</t>
         </is>
       </c>
       <c r="C7" s="8" t="n"/>
       <c r="D7" s="8" t="n"/>
     </row>
-    <row r="8" ht="42" customHeight="1">
+    <row r="8" ht="46" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>호텔</t>
+          <t>④ 호텔 경험</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>15:00 셋업 조건에서 무대 설치·리허설 시간 확보 방안</t>
+          <t>그랜드 하얏트 서울 Grand Ballroom 직접 수행 경험(행사명·연도), 설치·철거 경험, 호텔 Encore와의 AV 협의 경험</t>
         </is>
       </c>
       <c r="C8" s="8" t="n"/>
       <c r="D8" s="8" t="n"/>
     </row>
-    <row r="9" ht="42" customHeight="1">
+    <row r="9" ht="46" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>호텔</t>
+          <t>④ 호텔 경험</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Encore 감독비 등 호텔 관련 외부 비용의 예상 규모와 견적 반영 방식</t>
+          <t>15:00 셋업 조건에서 무대 설치·리허설 시간 확보 방안, Encore 감독비 등 호텔 관련 외부 비용의 예상 규모</t>
         </is>
       </c>
       <c r="C9" s="8" t="n"/>
       <c r="D9" s="8" t="n"/>
     </row>
-    <row r="10" ht="42" customHeight="1">
+    <row r="10" ht="46" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>등록</t>
+          <t>⑤ 프로그램</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>동문회 홈페이지(snubusiness.com) RSVP·QR 등록 연계 방식, 참석자 개인정보 처리</t>
+          <t>창립총회 의결·만찬·특별 강연·창립 세리머니·네트워킹을 18:00–21:00 안에 어떻게 배분하는가 (분 단위 개요)</t>
         </is>
       </c>
       <c r="C10" s="8" t="n"/>
       <c r="D10" s="8" t="n"/>
     </row>
-    <row r="11" ht="42" customHeight="1">
+    <row r="11" ht="46" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>현장</t>
+          <t>⑤ 프로그램</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>VIP 의전·좌석·동선 및 안전 관리 개요</t>
+          <t>창립 메시지를 드러내는 오프닝·세리머니 핵심 아이디어 1~2개</t>
         </is>
       </c>
       <c r="C11" s="8" t="n"/>
       <c r="D11" s="8" t="n"/>
     </row>
-    <row r="12" ht="42" customHeight="1">
+    <row r="12" ht="46" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>필수 동의</t>
+          <t>⑥ 제작·외주</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>행사 60일 전 호텔 서면 통보 및 외부 설치물·전기 사전 승인 이행</t>
+          <t>오프닝 영상·무대·AV·공연·디자인 각각 사내 제작인지 외주인지, 외주라면 파트너사명과 재하도급(2차 외주) 여부</t>
         </is>
       </c>
       <c r="C12" s="8" t="n"/>
       <c r="D12" s="8" t="n"/>
     </row>
-    <row r="13" ht="42" customHeight="1">
+    <row r="13" ht="46" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>필수 동의</t>
+          <t>⑦ 등록·개인정보</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>제안서 기재 핵심 인력의 실제 투입 확약</t>
+          <t>동문회 홈페이지(snubusiness.com) RSVP·QR 등록 연계 방식, 자체 등록 시스템 여부, 참석자 개인정보 수집·보관·파기 방식</t>
         </is>
       </c>
       <c r="C13" s="8" t="n"/>
       <c r="D13" s="8" t="n"/>
     </row>
-    <row r="14" ht="42" customHeight="1">
+    <row r="14" ht="46" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>필수 동의</t>
+          <t>⑧ 예산·계약</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>부가세 포함 1억 3,000만원 상한 내 필수안 제출</t>
+          <t>부가세 포함 1억 3,000만원 안에서 기획·PM비 / 직접 제작비 / 외주비 / 관리비·수수료를 분리한 견적이 가능한가 (시트 5에 작성)</t>
         </is>
       </c>
       <c r="C14" s="8" t="n"/>
       <c r="D14" s="8" t="n"/>
+    </row>
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>현장</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>VIP 의전·좌석·동선 및 안전 관리 개요</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+    </row>
+    <row r="16" ht="46" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>필수 동의</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>행사 60일 전 호텔 서면 통보 및 외부 설치물·전기 사전 승인 이행</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+    </row>
+    <row r="17" ht="46" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>필수 동의</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>제안서 기재 핵심 인력의 실제 투입 확약</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+    </row>
+    <row r="18" ht="46" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>필수 동의</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>부가세 포함 1억 3,000만원 상한 내 필수안 제출</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1474,7 +1530,7 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C12:C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C16:C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"동의,협의 필요"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>